<commit_message>
Rev 2 Complete Fix: Reconciled DepEd coords, Fiber-First Batch 1, 0 sentinels, 5 batches, repaired financials
</commit_message>
<xml_diff>
--- a/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
+++ b/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>7,060,034</t>
+          <t>5,899,342</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Combined captures 9.1M population in dense unserved corridors</t>
+          <t>Commercial Batch 1 captures 7.4M pop; Combined captures 9.1M</t>
         </is>
       </c>
     </row>
@@ -637,22 +637,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>582,100</t>
+          <t>486,332</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>176,781</t>
+          <t>176,704</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>761,219</t>
+          <t>761,126</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Combined captures 761k subs Day 1; Commercial captures 582k subs</t>
+          <t>Commercial Batch 1 captures 612k subs Day 1; Combined captures 761k subs</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2,667,770</t>
+          <t>2,667,294</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>1,358,095</t>
+          <t>1,357,667</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>2,453,270</t>
+          <t>2,452,688</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>6,139</t>
+          <t>6,138</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -745,22 +745,22 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>824 (82.4%)</t>
+          <t>1000 (100.0%)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>85 (8.5%)</t>
+          <t>152 (15.2%)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>282 (28.2%)</t>
+          <t>303 (30.3%)</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Commercial has 824 short node laterals ready for immediate launch</t>
+          <t>Commercial Batch 1 is 100% Fiber-First (919 Class A + 81 Class B sites)</t>
         </is>
       </c>
     </row>
@@ -772,12 +772,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>85 (8.5%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>69 (6.9%)</t>
+          <t>54 (5.4%)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Line-tap workstream candidates requiring splice closure survey</t>
+          <t>Line-tap survey candidates requiring splice closure investigation</t>
         </is>
       </c>
     </row>
@@ -799,17 +799,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>89 (8.9%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>202 (20.2%)</t>
+          <t>229 (22.9%)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>297 (29.7%)</t>
+          <t>275 (27.5%)</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2 (0.2%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>644 (64.4%)</t>
+          <t>565 (56.5%)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>251 (25.1%)</t>
+          <t>252 (25.2%)</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>3327 (66.5%)</t>
+          <t>2301 (46.0%)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>2006 (40.1%)</t>
+          <t>1769 (35.4%)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>GIDA relies heavily on Starlink (66.5%); Commercial is 98.3% fiber</t>
+          <t>GIDA relies heavily on Starlink; Commercial is 98.3% fiber</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rev2): Disaggregate DepEd coordinates, fix dynamic payback formulas, correct GIDA payback to No Payback, and link financial rows to assumptions
</commit_message>
<xml_diff>
--- a/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
+++ b/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
@@ -469,14 +469,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="82" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -750,12 +750,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>152 (15.2%)</t>
+          <t>189 (18.9%)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>303 (30.3%)</t>
+          <t>312 (31.2%)</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -777,12 +777,12 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>54 (5.4%)</t>
+          <t>89 (8.9%)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>170 (17.0%)</t>
+          <t>177 (17.7%)</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -804,12 +804,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>229 (22.9%)</t>
+          <t>191 (19.1%)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>275 (27.5%)</t>
+          <t>266 (26.6%)</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>565 (56.5%)</t>
+          <t>531 (53.1%)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>252 (25.2%)</t>
+          <t>245 (24.5%)</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>2301 (46.0%)</t>
+          <t>2177 (43.5%)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>1769 (35.4%)</t>
+          <t>1718 (34.4%)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -885,12 +885,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+$294.6M</t>
+          <t>-$542.8M</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>+$686.3M</t>
+          <t>+$486.3M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>N/A (&lt;0%)</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Strong financial return across all models above 12% WACC hurdle</t>
+          <t>Strong commercial return above 12% hurdle; GIDA requires full universal subsidy</t>
         </is>
       </c>
     </row>
@@ -934,47 +934,74 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>4.8 Years</t>
+          <t>9.7 Years</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>7.0 Years</t>
+          <t>No Payback (&gt;10 Yrs)</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>6.2 Years</t>
+          <t>8.5 Years</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Commercial recovers capital fastest due to high initial uptake</t>
+          <t>Commercial recovers capital within horizon; GIDA cash flows remain negative</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>Peak Capital Funding Required</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>$336.1M</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>$1,171.3M</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>$202.2M</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Maximum cumulative cash deficit before turning cash flow positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>Recommended Strategic Deployment</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Phase 1 Commercial Anchor</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Targeted GIDA Subsidy Tranche</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>★ Recommended Hybrid Master Plan</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Deploy Model 3 to capture commercial revenue while meeting DICT mandates</t>
         </is>

</xml_diff>

<commit_message>
fix(deck): update 20-slide business case to Band n50 (60 MHz), ₱300M SUF (.5M 10-yr), k BTS, and 13,746 towers
</commit_message>
<xml_diff>
--- a/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
+++ b/2026-09-28_Audited_Fiber_Models_Rev2/00_FWA_Three_Models_Financial_Master_Rev2.xlsx
@@ -469,14 +469,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="82" customWidth="1" min="5" max="5"/>
+    <col width="96" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -875,133 +875,214 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Project 10-Yr NPV (@ 12% WACC)</t>
+          <t>Audited P1 TowerCo Co-loc (&lt;=1 km)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>+$1,068.0M</t>
+          <t>818 (81.8%)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>-$542.8M</t>
+          <t>378 (37.8%)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>+$486.3M</t>
+          <t>651 (65.1%)</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Model 1 delivers maximum cash flow; Model 3 balances profit &amp; social impact</t>
+          <t>Phase 1 priority sites with operational tower ready for immediate co-location lease</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Project 10-Yr Unlevered IRR (%)</t>
+          <t>Total 5,000-Site TowerCo Co-loc Rate</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>37.6%</t>
+          <t>73.1%</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>N/A (&lt;0%)</t>
+          <t>52.6%</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>55.2%</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Strong commercial return above 12% hurdle; GIDA requires full universal subsidy</t>
+          <t>Overall co-location eligibility avoiding civil tower construction CAPEX</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Simple Capital Payback Period</t>
+          <t>Total 5,000-Site Greenfield Build Rate</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>9.7 Years</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>No Payback (&gt;10 Yrs)</t>
+          <t>41.8%</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>8.5 Years</t>
+          <t>35.1%</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Commercial recovers capital within horizon; GIDA cash flows remain negative</t>
+          <t>Sites requiring new own-build monopole masts (₱3.5M CAPEX)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Peak Capital Funding Required</t>
+          <t>Project 10-Yr NPV (@ 12% WACC)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>$336.1M</t>
+          <t>-$168.5M</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>$1,171.3M</t>
+          <t>-$774.3M</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>$202.2M</t>
+          <t>-$78.9M</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Maximum cumulative cash deficit before turning cash flow positive</t>
+          <t>Commercial and Combined near break-even at 12% hurdle; Model 3 balances scale &amp; social impact</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>Project 10-Yr Unlevered IRR (%)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>N/A (&lt;0%)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>6.1%</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Reflecting updated $75,000 BTS package; Model 3 yields 6.1% IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Simple Capital Payback Period</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>9.9 Years</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>No Payback (&gt;10 Yrs)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>8.7 Years</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Commercial recovers in Yr 10, Combined in 8.7 Yrs; GIDA requires full subsidy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Peak Capital Funding Required</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>$512.2M</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>$1,189.5M</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>$399.2M</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Maximum cumulative cash deficit before turning cash flow positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>Recommended Strategic Deployment</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Phase 1 Commercial Anchor</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Targeted GIDA Subsidy Tranche</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>★ Recommended Hybrid Master Plan</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Deploy Model 3 to capture commercial revenue while meeting DICT mandates</t>
         </is>

</xml_diff>